<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@9cd58254fce717b60b78f2c11b935ab5b405b500 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-ICD10dut.xlsx
+++ b/CodeSystem-ICD10dut.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>Property</t>
   </si>
@@ -77,7 +77,10 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>No display for ContactDetail</t>
+    <t>RIVO-NN (https://rivo-noord.nl)</t>
+  </si>
+  <si>
+    <t>HL7NL (https://hl7.nl)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -359,86 +362,86 @@
         <v>20</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24" s="2"/>
     </row>

</xml_diff>